<commit_message>
made users a dropdown + made all dropdowns in all pages to close once you click on the object again + made view all and edit with all the fields the client wanted in the pdf file he sent us and all the fields from the excel + excel seed is being fully imported and working (still need more tests) + streets seed is fully functional and working + made the fields they wanted to be tables exactly as they wanted and exatcly the same selected options + made view all and edit buildigns fields to be ordered the same in the frontend + added sorting in users and street page #11 + # 16 + #41
</commit_message>
<xml_diff>
--- a/project/web-server/backend/Data/BuildingsSeedData.xlsx
+++ b/project/web-server/backend/Data/BuildingsSeedData.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="2390" documentId="11_095C25CF7C08AC45DA151025DDBF931F85697602" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6295D60B-0E62-4563-BD9C-8ADB4928959C}"/>
+  <xr:revisionPtr revIDLastSave="2394" documentId="11_095C25CF7C08AC45DA151025DDBF931F85697602" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8349B9B8-C835-4E69-B633-82697908D81C}"/>
   <bookViews>
     <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4584,10 +4584,10 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="5" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -4618,6 +4618,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -5117,94 +5121,94 @@
       <c r="L2" s="1"/>
       <c r="M2" s="1"/>
       <c r="N2" s="1"/>
-      <c r="O2" s="46" t="s">
+      <c r="O2" s="45" t="s">
         <v>3</v>
       </c>
-      <c r="P2" s="46"/>
-      <c r="Q2" s="46"/>
-      <c r="R2" s="46"/>
-      <c r="S2" s="46"/>
-      <c r="T2" s="46"/>
-      <c r="U2" s="46"/>
-      <c r="V2" s="46"/>
-      <c r="W2" s="46"/>
-      <c r="X2" s="46"/>
-      <c r="Y2" s="46"/>
-      <c r="Z2" s="46"/>
-      <c r="AA2" s="46"/>
-      <c r="AB2" s="46"/>
-      <c r="AC2" s="46"/>
-      <c r="AD2" s="46"/>
-      <c r="AE2" s="46"/>
-      <c r="AF2" s="46"/>
-      <c r="AG2" s="46"/>
-      <c r="AH2" s="45" t="s">
+      <c r="P2" s="45"/>
+      <c r="Q2" s="45"/>
+      <c r="R2" s="45"/>
+      <c r="S2" s="45"/>
+      <c r="T2" s="45"/>
+      <c r="U2" s="45"/>
+      <c r="V2" s="45"/>
+      <c r="W2" s="45"/>
+      <c r="X2" s="45"/>
+      <c r="Y2" s="45"/>
+      <c r="Z2" s="45"/>
+      <c r="AA2" s="45"/>
+      <c r="AB2" s="45"/>
+      <c r="AC2" s="45"/>
+      <c r="AD2" s="45"/>
+      <c r="AE2" s="45"/>
+      <c r="AF2" s="45"/>
+      <c r="AG2" s="45"/>
+      <c r="AH2" s="46" t="s">
         <v>8</v>
       </c>
-      <c r="AI2" s="45"/>
-      <c r="AJ2" s="45"/>
-      <c r="AK2" s="45"/>
-      <c r="AL2" s="45"/>
-      <c r="AM2" s="45"/>
-      <c r="AN2" s="45"/>
-      <c r="AO2" s="46" t="s">
+      <c r="AI2" s="46"/>
+      <c r="AJ2" s="46"/>
+      <c r="AK2" s="46"/>
+      <c r="AL2" s="46"/>
+      <c r="AM2" s="46"/>
+      <c r="AN2" s="46"/>
+      <c r="AO2" s="45" t="s">
         <v>23</v>
       </c>
-      <c r="AP2" s="46"/>
-      <c r="AQ2" s="45" t="s">
+      <c r="AP2" s="45"/>
+      <c r="AQ2" s="46" t="s">
         <v>31</v>
       </c>
-      <c r="AR2" s="45"/>
-      <c r="AS2" s="45"/>
-      <c r="AT2" s="45"/>
-      <c r="AU2" s="45"/>
-      <c r="AV2" s="45"/>
-      <c r="AW2" s="45"/>
-      <c r="AX2" s="45"/>
-      <c r="AY2" s="45"/>
-      <c r="AZ2" s="45"/>
-      <c r="BA2" s="45"/>
+      <c r="AR2" s="46"/>
+      <c r="AS2" s="46"/>
+      <c r="AT2" s="46"/>
+      <c r="AU2" s="46"/>
+      <c r="AV2" s="46"/>
+      <c r="AW2" s="46"/>
+      <c r="AX2" s="46"/>
+      <c r="AY2" s="46"/>
+      <c r="AZ2" s="46"/>
+      <c r="BA2" s="46"/>
       <c r="BB2" s="47"/>
       <c r="BC2" s="47"/>
-      <c r="BD2" s="45"/>
-      <c r="BE2" s="45"/>
-      <c r="BF2" s="46"/>
-      <c r="BG2" s="46"/>
-      <c r="BH2" s="46"/>
-      <c r="BI2" s="46"/>
-      <c r="BJ2" s="46"/>
-      <c r="BK2" s="46"/>
-      <c r="BL2" s="45" t="s">
+      <c r="BD2" s="46"/>
+      <c r="BE2" s="46"/>
+      <c r="BF2" s="45"/>
+      <c r="BG2" s="45"/>
+      <c r="BH2" s="45"/>
+      <c r="BI2" s="45"/>
+      <c r="BJ2" s="45"/>
+      <c r="BK2" s="45"/>
+      <c r="BL2" s="46" t="s">
         <v>42</v>
       </c>
-      <c r="BM2" s="45"/>
-      <c r="BN2" s="45"/>
-      <c r="BO2" s="46" t="s">
+      <c r="BM2" s="46"/>
+      <c r="BN2" s="46"/>
+      <c r="BO2" s="45" t="s">
         <v>47</v>
       </c>
-      <c r="BP2" s="46"/>
-      <c r="BQ2" s="46"/>
-      <c r="BR2" s="46"/>
-      <c r="BS2" s="46"/>
-      <c r="BT2" s="46"/>
-      <c r="BU2" s="45" t="s">
+      <c r="BP2" s="45"/>
+      <c r="BQ2" s="45"/>
+      <c r="BR2" s="45"/>
+      <c r="BS2" s="45"/>
+      <c r="BT2" s="45"/>
+      <c r="BU2" s="46" t="s">
         <v>54</v>
       </c>
-      <c r="BV2" s="45"/>
-      <c r="BW2" s="45"/>
-      <c r="BX2" s="45"/>
-      <c r="BY2" s="46" t="s">
+      <c r="BV2" s="46"/>
+      <c r="BW2" s="46"/>
+      <c r="BX2" s="46"/>
+      <c r="BY2" s="45" t="s">
         <v>61</v>
       </c>
-      <c r="BZ2" s="46"/>
-      <c r="CA2" s="46"/>
-      <c r="CB2" s="46"/>
-      <c r="CC2" s="46"/>
-      <c r="CD2" s="45" t="s">
+      <c r="BZ2" s="45"/>
+      <c r="CA2" s="45"/>
+      <c r="CB2" s="45"/>
+      <c r="CC2" s="45"/>
+      <c r="CD2" s="46" t="s">
         <v>1317</v>
       </c>
-      <c r="CE2" s="45"/>
-      <c r="CF2" s="45"/>
+      <c r="CE2" s="46"/>
+      <c r="CF2" s="46"/>
     </row>
     <row r="3" spans="1:84" ht="51.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="30" t="s">
@@ -5892,16 +5896,16 @@
     <sortCondition ref="G4:G6"/>
   </sortState>
   <mergeCells count="10">
+    <mergeCell ref="CD2:CF2"/>
+    <mergeCell ref="BL2:BN2"/>
+    <mergeCell ref="BO2:BT2"/>
+    <mergeCell ref="BU2:BX2"/>
+    <mergeCell ref="BY2:CC2"/>
     <mergeCell ref="O2:AG2"/>
     <mergeCell ref="AH2:AN2"/>
     <mergeCell ref="AO2:AP2"/>
     <mergeCell ref="AQ2:BE2"/>
     <mergeCell ref="BF2:BK2"/>
-    <mergeCell ref="CD2:CF2"/>
-    <mergeCell ref="BL2:BN2"/>
-    <mergeCell ref="BO2:BT2"/>
-    <mergeCell ref="BU2:BX2"/>
-    <mergeCell ref="BY2:CC2"/>
   </mergeCells>
   <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>

</xml_diff>